<commit_message>
Đối chiếu 74 nghiệp vụ với mã hiện có: đủ 36 · một phần 24 · chưa 13
Cột đáng chú ý nhất không phải 'đã làm hay chưa' mà là khoảng cách giữa mức tự
chủ ĐỀ XUẤT và mức ĐẠT ĐƯỢC: 29/74 việc đang chạy thấp hơn thiết kế. Cơ chế thì
đủ, phần CHỦ ĐỘNG thì thiếu.

Hai giai đoạn đầu gần như trống về tự chủ: GĐ0 (0 đủ / 6) và GĐ4 (0 đủ / 4) —
đều là chỗ Agent phải HỎI và ĐỀ XUẤT. Hai giai đoạn mạnh nhất là GĐ2 (5/5) và
GĐ5 (7/8) — đều là chỗ có đầu vào rõ và chỉ cần thi hành.

Ghi nhận trung thực một mục: N-905 (ghi nhận sai lệch thiết kế) tuy có nhật ký
40 mục nhưng do tôi ghi tay, Agent không tự phát hiện — nên đạt T0 chứ không T3.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkergxFj3g4rz31wprC4ZP
</commit_message>
<xml_diff>
--- a/docs/EAA_Nghiep_vu_Agent.xlsx
+++ b/docs/EAA_Nghiep_vu_Agent.xlsx
@@ -11,9 +11,11 @@
     <sheet name="Nghiệp vụ" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Câu hỏi phải biết hỏi" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Thống kê" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Đối chiếu" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Nghiệp vụ'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Đối chiếu'!$A$1:$I$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +56,24 @@
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +115,26 @@
         <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,6 +220,43 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4618,7 +4693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4999,7 +5074,3801 @@
         <v>13</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="22" t="n"/>
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="22" t="n"/>
+      <c r="G16" s="22" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Đối chiếu với mã hiện có</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="n"/>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="22" t="n"/>
+      <c r="G17" s="22" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Việc</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>Cố ý không</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
+        <is>
+          <t>Có khoảng cách tự chủ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="22" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>GĐ2 · Môi trường &amp; công cụ</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>GĐ4 · Thiết kế &amp; phân rã</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>GĐ6 · Mô phỏng</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>GĐ9 · Nghiệm thu &amp; phát hành</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>GĐ10 · Vận hành &amp; bảo trì</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n">
+        <v>74</v>
+      </c>
+      <c r="C31" s="25" t="n">
+        <v>36</v>
+      </c>
+      <c r="D31" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="F31" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="25" t="n">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="66" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Mã</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Giai đoạn</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Nghiệp vụ</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Tự chủ
+ĐỀ XUẤT</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Tự chủ
+ĐẠT</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Khoảng
+cách</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Bằng chứng trong mã</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Còn thiếu gì</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>N-001</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp nhận yêu cầu bằng lời của người dùng</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G2" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Không có lệnh nào tiếp nhận yêu cầu. Người tự viết constraints.yaml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>N-002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Dò phần cứng đang cắm vào máy</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E3" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F3" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G3" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>eaa/serialport.py + eaa ports · TC-42a</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Chưa đọc ổ mass-storage của mạch nạp; chưa có danh mục bo để tra VID/PID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>N-003</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Nhận dạng bo/MCU từ dấu hiệu dò được</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Chỉ so với VID/PID mà DỰ ÁN tự khai. Không có danh mục bo, không đề xuất ứng viên, không hỏi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>N-004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Thu thập tài liệu gốc</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>eaa/ingest.py (PdfIngestor, check_web_source) · TC-22</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Không liệt kê đích danh tài liệu cần; không hỏi rev silicon; không hỏi errata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>N-005</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Lập danh mục giả định ban đầu</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>eaa/ingest.py AssumptionLog · TC-22</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Có kho giả định, nhưng danh mục ban đầu do người viết tay (hồ sơ DISCO là tôi gõ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>N-006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>GĐ0 · Tiếp nhận &amp; phạm vi</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Xác định phạm vi và cái KHÔNG làm</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Không có bước chốt phạm vi và cái không làm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>N-010</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Chốt ràng buộc cứng</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>eaa/kb.py Constraints + G1 · TC-04</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Đọc/kiểm/duyệt được, nhưng Agent KHÔNG đề xuất bộ ràng buộc — người viết trước.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>N-011</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Định nghĩa tiêu chí nghiệm thu ĐO ĐƯỢC</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>eaa/acceptance.py · TC-45</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Đối chiếu tiêu chí thì đủ; Agent không đề xuất tiêu chí và không ép 'phải đo được'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>N-012</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Chọn kiến trúc phần mềm</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>eaa/options.py + eaa decide · TC-46</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>N-013</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Phân bổ tài nguyên phần cứng</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>eaa/graph.py check_module · TC-18</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>N-014</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Chốt sơ đồ chân</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>hardware_profile.yaml → graph · TC-18</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Đọc được pin_map; không trích từ schematic, không đề xuất, không kiểm chân có hỗ trợ chức năng cần.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>N-015</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Lập ngân sách tài nguyên</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>constraints.limits + SizeGate · TC-40d</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm được TỔNG; không chia ngân sách theo module, không cảnh báo module ăn quá phần.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>N-016</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Phân tích hỏng hóc và hệ quả</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Không có phân tích hỏng hóc–hệ quả.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>N-017</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>GĐ1 · Phân tích &amp; đặc tả</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Xác định chế độ an toàn</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G15" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Không có định nghĩa chế độ an toàn. (safety_checklist chỉ dành cho kịch bản chẩn đoán, khác việc này.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>N-020</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>GĐ2 · Môi trường &amp; công cụ</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm công cụ đã có trên máy</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F16" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G16" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>eaa/doctor.py + toolsearch.derive_requirements · TC-34, TC-39</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>N-021</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>GĐ2 · Môi trường &amp; công cụ</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Tìm công cụ chưa biết cách cài</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>eaa/toolsearch.py · TC-39</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>N-022</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>GĐ2 · Môi trường &amp; công cụ</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Cài công cụ</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E18" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F18" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>eaa doctor --fix · TC-34, TC-37</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>N-023</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>GĐ2 · Môi trường &amp; công cụ</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Khóa phiên bản môi trường</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F19" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>eaa/doctor.py EnvLock · TC-36</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>N-024</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>GĐ2 · Môi trường &amp; công cụ</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Dựng kho mã và quy ước commit</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F20" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>eaa/vcs.py · TC-01</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>N-030</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Chọn trang tài liệu cần trích</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G21" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>eaa datasheet ingest · TC-22</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Người chọn trang (đúng thiết kế), nhưng Agent không nêu ĐÍCH DANH trang cần trích.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>N-031</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Chưng cất trích đoạn thành bảng thanh ghi–bit</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E22" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F22" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>eaa/ingest.py → G2 · TC-22</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>N-032</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Dựng đồ thị tri thức</t>
+        </is>
+      </c>
+      <c r="D23" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E23" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F23" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G23" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>eaa/graph.py · TC-18</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>N-033</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Phát hiện mâu thuẫn nguồn</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>eaa/readiness.py conflict + chuẩn hóa số · TC-26</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>N-034</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Tự đánh giá đủ thông tin trước khi sinh mã</t>
+        </is>
+      </c>
+      <c r="D25" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G25" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>eaa/readiness.py · TC-24</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>N-035</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Đi tìm thứ còn thiếu (leo thang 3 bậc)</t>
+        </is>
+      </c>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E26" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G26" s="29" t="inlineStr">
+        <is>
+          <t>−2</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>eaa/gapsearch.py (WIP, chưa nối CLI, chưa test)</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Hiện hành: chỉ IN GỢI Ý ba bậc rồi dừng. search_rounds không ai tăng. Chưa đi tìm thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>N-036</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Quản lý vòng đời tri thức</t>
+        </is>
+      </c>
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E27" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F27" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G27" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>eaa/lifecycle.py (3 đường truy ngược) · TC-29</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>N-037</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>GĐ3 · Tri thức phần cứng</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Theo dõi errata của nhà sản xuất</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G28" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Không hỏi rev silicon, không tra errata, không đối chiếu với ngoại vi đang dùng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>N-040</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4 · Thiết kế &amp; phân rã</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Phân rã bài toán thành module</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F29" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G29" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>eaa plan add (thủ công)</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Agent không đề xuất phân rã. Người tự liệt kê module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>N-041</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4 · Thiết kế &amp; phân rã</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Định nghĩa giao diện giữa module</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E30" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G30" s="29" t="inlineStr">
+        <is>
+          <t>−2</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>eaa/composer.py lớp K3</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Đọc được tệp tiêu đề module đã merge; KHÔNG sinh interface trước khi sinh thân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>N-042</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4 · Thiết kế &amp; phân rã</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Xếp thứ tự làm theo phụ thuộc</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E31" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F31" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G31" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>state.BacklogItem.depends_on · TC-18</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Dùng để nạp interface và kiểm xung đột; không sắp thứ tự topo, không tự chọn module kế tiếp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>N-043</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>GĐ4 · Thiết kế &amp; phân rã</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Thiết kế lịch chạy</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F32" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G32" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>projects/*/firmware.yaml · TC-41a</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm được chu kỳ hợp lệ; Agent không đề xuất chu kỳ, không ước lượng tải CPU, không cảnh báo quá tải.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>N-050</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Sinh mã một module</t>
+        </is>
+      </c>
+      <c r="D33" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E33" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F33" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G33" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>eaa/composer.py + orchestrator · TC-04, TC-17</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>N-051</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Biên dịch</t>
+        </is>
+      </c>
+      <c r="D34" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E34" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F34" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G34" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>eaa/tools/compile.py CompileGate · TC-40</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>N-052</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Phân tích tĩnh theo ràng buộc dự án</t>
+        </is>
+      </c>
+      <c r="D35" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E35" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F35" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G35" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>eaa/tools/static.py · TC-07</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>N-053</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm thử đơn vị trên máy chủ</t>
+        </is>
+      </c>
+      <c r="D36" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E36" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F36" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G36" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>eaa/tools/unittests.py · TC-07</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Chạy được; không nêu rõ phần nào KHÔNG kiểm được trên máy chủ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>N-054</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Đo chiếm dụng bộ nhớ</t>
+        </is>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E37" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G37" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>eaa/tools/compile.py SizeGate + size_scope · TC-40d</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>N-055</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Vòng tự sửa khi cổng không đạt</t>
+        </is>
+      </c>
+      <c r="D38" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F38" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G38" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>eaa/orchestrator.py · TC-06, TC-19</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>N-056</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Review và hợp nhất</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E39" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F39" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G39" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>eaa/gates.py + vcs.py content_digest · TC-01</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>N-057</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>GĐ5 · Sinh mã &amp; kiểm chứng tĩnh</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Ghi nhận lỗi mô hình bịa ra</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E40" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F40" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G40" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>eaa/ledger.py · TC-10</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>N-060</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6 · Mô phỏng</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Dựng mô hình đối tượng điều khiển</t>
+        </is>
+      </c>
+      <c r="D41" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F41" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G41" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>projects/robot_balance/sim/</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Dự án mẫu có mô hình con lắc; Agent không đề xuất mô hình cho đối tượng mới.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>N-061</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6 · Mô phỏng</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Chạy mô phỏng vòng kín</t>
+        </is>
+      </c>
+      <c r="D42" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E42" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F42" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G42" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>eaa/tools/sim.py, sim_runner.py · TC-12</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>N-062</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6 · Mô phỏng</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Quét tham số và đề xuất bộ tham số</t>
+        </is>
+      </c>
+      <c r="D43" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G43" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>eaa sim --sweep · TC-12</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>N-063</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6 · Mô phỏng</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Tiêm lỗi trong mô phỏng</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E44" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F44" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G44" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>Không tiêm lỗi trong mô phỏng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>N-064</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>GĐ6 · Mô phỏng</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Chạy chính mã C sinh ra trong mô phỏng</t>
+        </is>
+      </c>
+      <c r="D45" s="36" t="inlineStr">
+        <is>
+          <t>Cố ý không làm</t>
+        </is>
+      </c>
+      <c r="E45" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F45" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G45" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Cố ý để ngoài chuỗi tự động: nối vào mà không thật sự chạy artifact thì cổng sẽ 'đạt' mà chẳng kiểm gì.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>N-070</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Ráp firmware hoàn chỉnh</t>
+        </is>
+      </c>
+      <c r="D46" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E46" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F46" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G46" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>eaa/firmware.py + eaa build · TC-41</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>N-071</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm bộ nhớ ở tầm firmware</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E47" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F47" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G47" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>SizeGate scope=firmware · TC-41e</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Đo được flash/RAM ở tầm firmware; KHÔNG kiểm khoảng trống ngăn xếp còn lại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>N-072</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm trước khi nạp</t>
+        </is>
+      </c>
+      <c r="D48" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E48" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F48" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G48" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>eaa/flash.py preflight · TC-42b</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>N-073</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Chọn đúng thiết bị để nạp</t>
+        </is>
+      </c>
+      <c r="D49" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E49" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F49" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G49" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>eaa/serialport.py match_confirmed · TC-47d</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>N-074</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Nạp và ghi nhật ký</t>
+        </is>
+      </c>
+      <c r="D50" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E50" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F50" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G50" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>eaa/flash.py + FlashLog · TC-42d</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>N-075</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>GĐ7 · Ráp &amp; nạp</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm sau khi nạp</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E51" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F51" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G51" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>Không đọc ngược/so kiểm tổng sau khi nạp. 'Nạp không báo lỗi' đang bị ngầm hiểu là 'nạp đúng'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>N-080</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Thiết lập kênh đo</t>
+        </is>
+      </c>
+      <c r="D52" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E52" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F52" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G52" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>eaa/telemetry.py + eaa telemetry · TC-43</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>N-081</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Sinh firmware đo cho từng kịch bản chẩn đoán</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E53" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F53" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G53" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>eaa/firmware.py DiagnosticFirmwareBuilder · TC-44</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>Cơ chế đủ; mới 2/6 kịch bản có phần đo (DS-01, DS-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>N-082</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Chẩn đoán hai kênh</t>
+        </is>
+      </c>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F54" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G54" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>eaa/diagnostics.py · TC-27</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>N-083</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Đo đặc tính thời gian thực</t>
+        </is>
+      </c>
+      <c r="D55" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E55" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F55" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G55" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>acceptance loop_period_ms + telemetry</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>Có kênh và có tiêu chí; CHƯA có firmware đo dao động chu kỳ và tải CPU, chưa báo trường hợp xấu nhất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>N-084</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Đo điện và nhiệt</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E56" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="F56" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G56" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>diagnostics.yaml DS-05 (mới khai, chưa có phần đo)</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Không có hướng dẫn đo đích danh, không có chỗ nhập số đo tay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>N-085</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Chẩn đoán sâu bằng công cụ gỡ lỗi</t>
+        </is>
+      </c>
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E57" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F57" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G57" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi đề án (đã ghi từ trước).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>N-086</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>GĐ8 · Đưa lên mạch &amp; đo</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Kiểm độ bền dài hạn</t>
+        </is>
+      </c>
+      <c r="D58" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E58" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F58" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G58" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>acceptance uptime_s ≥ 600 · TC-45</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Có tiêu chí; không có cơ chế chạy dài, không phát hiện reset qua bộ đếm thời gian chạy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>N-090</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>GĐ9 · Nghiệm thu &amp; phát hành</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Đối chiếu tiêu chí nghiệm thu</t>
+        </is>
+      </c>
+      <c r="D59" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E59" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F59" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G59" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>eaa/acceptance.py · TC-45</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>N-091</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>GĐ9 · Nghiệm thu &amp; phát hành</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Phong hạng chất lượng bản mã</t>
+        </is>
+      </c>
+      <c r="D60" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E60" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F60" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G60" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>eaa/versions.py + check_device_commit · TC-30, TC-45a</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>N-092</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>GĐ9 · Nghiệm thu &amp; phát hành</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Giữ bản chạy tốt và quay lui</t>
+        </is>
+      </c>
+      <c r="D61" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E61" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F61" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G61" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>eaa/versions.py + eaa rollback · TC-30</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>N-093</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>GĐ9 · Nghiệm thu &amp; phát hành</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Xuất báo cáo và dấu vết</t>
+        </is>
+      </c>
+      <c r="D62" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E62" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F62" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G62" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>eaa/kpi.py + llm/calllog.py + registry.py · TC-09, TC-15</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>N-094</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>GĐ9 · Nghiệm thu &amp; phát hành</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Bàn giao tài liệu vận hành</t>
+        </is>
+      </c>
+      <c r="D63" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F63" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G63" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>eaa/registry.py (kho phẩm xuất) · TC-32</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>Lưu/gửi lại phẩm xuất được; KHÔNG sinh tài liệu vận hành từ dữ liệu dự án.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>N-100</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>GĐ10 · Vận hành &amp; bảo trì</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Đánh giá ảnh hưởng khi tài liệu đổi</t>
+        </is>
+      </c>
+      <c r="D64" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E64" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F64" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G64" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>eaa/lifecycle.py · TC-29</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>N-101</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>GĐ10 · Vận hành &amp; bảo trì</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Đánh giá ảnh hưởng khi linh kiện đổi</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E65" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F65" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G65" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>Không so sánh linh kiện thay thế.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>N-102</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>GĐ10 · Vận hành &amp; bảo trì</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Chẩn đoán sự cố ngoài hiện trường</t>
+        </is>
+      </c>
+      <c r="D66" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F66" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="G66" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>eaa diagnose select + hai kênh · TC-27</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>Chọn kịch bản từ triệu chứng được; không dựng lại điều kiện sự cố, không xử lý ca không tái hiện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>N-103</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>GĐ10 · Vận hành &amp; bảo trì</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Cập nhật firmware cho thiết bị đã triển khai</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="inlineStr">
+        <is>
+          <t>Chưa có</t>
+        </is>
+      </c>
+      <c r="E67" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F67" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G67" s="29" t="inlineStr">
+        <is>
+          <t>−2</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>Không có cập nhật firmware cho thiết bị đã triển khai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>N-900</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Giữ ranh giới tổng quát / nền tảng / dự án</t>
+        </is>
+      </c>
+      <c r="D68" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E68" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F68" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G68" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>TC-38 (quét mỗi commit) + TC-47a (không rẽ nhánh theo pack)</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>N-901</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Bảo vệ khóa và bí mật</t>
+        </is>
+      </c>
+      <c r="D69" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E69" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F69" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G69" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>eaa/llm/base.py mask_secrets · TC-14 + tests/conftest.py</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>N-902</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Không bao giờ hành động ngoài ý muốn người</t>
+        </is>
+      </c>
+      <c r="D70" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E70" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F70" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>eaa/gates.py, doctor, flash — không cờ bỏ qua · TC-01, TC-42c</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>N-903</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Nói rõ mức tin cậy của mọi điều mình nói</t>
+        </is>
+      </c>
+      <c r="D71" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E71" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F71" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G71" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>serialport.match_confirmed, telemetry.bad_ratio, AssumptionLog</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Có ở vài chỗ; CHƯA nhất quán toàn hệ — nhiều đầu ra không nói mức tin cậy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>N-904</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Quản lý chi phí gọi mô hình</t>
+        </is>
+      </c>
+      <c r="D72" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E72" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F72" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>eaa/kpi.py (tokens_in/out) · TC-09</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>Ghi được token; không có trần theo module, không quy ra chi phí, không cảnh báo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>N-905</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Ghi nhận mọi sai lệch so với thiết kế</t>
+        </is>
+      </c>
+      <c r="D73" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E73" s="33" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F73" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G73" s="29" t="inlineStr">
+        <is>
+          <t>−3</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>docs/SAI_LECH_THIET_KE.md (40 mục)</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>Nhật ký đầy đủ, nhưng do TÔI ghi tay — Agent không tự phát hiện và không tự ghi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>N-906</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Tự đánh giá và cải tiến quy trình</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="inlineStr">
+        <is>
+          <t>Một phần</t>
+        </is>
+      </c>
+      <c r="E74" s="27" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F74" s="28" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="G74" s="29" t="inlineStr">
+        <is>
+          <t>−1</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>eaa report + kpi.summary · TC-09</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>Tổng hợp được chỉ số; không chỉ ra khâu hay hỏng, không đề xuất sửa prompt/quy tắc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>N-907</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>XS · Xuyên suốt</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Khôi phục sau gián đoạn</t>
+        </is>
+      </c>
+      <c r="D75" s="34" t="inlineStr">
+        <is>
+          <t>Đủ</t>
+        </is>
+      </c>
+      <c r="E75" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="F75" s="31" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="G75" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>eaa/state.py ghi nguyên tử + eaa resume · TC-03</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I75"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>